<commit_message>
content: add sourcing note to France Bioinformatics entries in coverage_matrix.xlsx
</commit_message>
<xml_diff>
--- a/research/long-bet/raw/coverage_matrix.xlsx
+++ b/research/long-bet/raw/coverage_matrix.xlsx
@@ -351,7 +351,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -373,11 +373,55 @@
         <color rgb="00E2E8F0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -687,6 +731,8 @@
     <xf numFmtId="0" fontId="17" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -761,6 +807,31 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Fix Instructions - Item 1</author>
+  </authors>
+  <commentList>
+    <comment ref="AD16" authorId="0" shapeId="0">
+      <text>
+        <t>Verified July 2026: provision is via undergraduate double licence (maths/CS + biology) feeding a specialised Master's, not a standalone UG Bioinformatics degree. Confirmed for Paris-Saclay, Sorbonne, and Universite Paris Cite. Article 3 France section updated to reflect this. Licence-level teaching is in French.</t>
+      </text>
+    </comment>
+    <comment ref="AD46" authorId="0" shapeId="0">
+      <text>
+        <t>Verified July 2026: provision is via undergraduate double licence (maths/CS + biology) feeding a specialised Master's, not a standalone UG Bioinformatics degree. Confirmed for Paris-Saclay, Sorbonne, and Universite Paris Cite. Article 3 France section updated to reflect this. Licence-level teaching is in French.</t>
+      </text>
+    </comment>
+    <comment ref="AD63" authorId="0" shapeId="0">
+      <text>
+        <t>Verified July 2026: provision is via undergraduate double licence (maths/CS + biology) feeding a specialised Master's, not a standalone UG Bioinformatics degree. Confirmed for Paris-Saclay, Sorbonne, and Universite Paris Cite. Article 3 France section updated to reflect this. Licence-level teaching is in French.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1114,21 +1185,31 @@
           <t>CS &amp; AI</t>
         </is>
       </c>
+      <c r="E1" s="105" t="n"/>
+      <c r="F1" s="105" t="n"/>
+      <c r="G1" s="105" t="n"/>
+      <c r="H1" s="106" t="n"/>
       <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
+      <c r="J1" s="105" t="n"/>
+      <c r="K1" s="105" t="n"/>
+      <c r="L1" s="105" t="n"/>
+      <c r="M1" s="106" t="n"/>
       <c r="N1" s="4" t="inlineStr">
         <is>
           <t>Physics &amp; Astronomy</t>
         </is>
       </c>
+      <c r="O1" s="106" t="n"/>
       <c r="P1" s="5" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
+      <c r="Q1" s="106" t="n"/>
       <c r="R1" s="6" t="inlineStr">
         <is>
           <t>Engineering – Electrical &amp; Computer</t>
@@ -1139,16 +1220,19 @@
           <t>Engineering – Mechanical &amp; Aerospace</t>
         </is>
       </c>
+      <c r="T1" s="106" t="n"/>
       <c r="U1" s="8" t="inlineStr">
         <is>
           <t>Engineering – Civil &amp; Environmental</t>
         </is>
       </c>
+      <c r="V1" s="106" t="n"/>
       <c r="W1" s="9" t="inlineStr">
         <is>
           <t>Engineering – Chemical &amp; Materials</t>
         </is>
       </c>
+      <c r="X1" s="106" t="n"/>
       <c r="Y1" s="10" t="inlineStr">
         <is>
           <t>Engineering – Biomedical</t>
@@ -1159,11 +1243,16 @@
           <t>Engineering – Other</t>
         </is>
       </c>
+      <c r="AA1" s="105" t="n"/>
+      <c r="AB1" s="105" t="n"/>
+      <c r="AC1" s="106" t="n"/>
       <c r="AD1" s="12" t="inlineStr">
         <is>
           <t>Computational Biology &amp; Bioinformatics</t>
         </is>
       </c>
+      <c r="AE1" s="105" t="n"/>
+      <c r="AF1" s="106" t="n"/>
       <c r="AG1" s="13" t="inlineStr">
         <is>
           <t>Earth &amp; Environmental Sciences</t>
@@ -17855,8 +17944,8 @@
   <mergeCells count="12">
     <mergeCell ref="B1"/>
     <mergeCell ref="AD1:AF1"/>
+    <mergeCell ref="S1:T1"/>
     <mergeCell ref="D1:H1"/>
-    <mergeCell ref="S1:T1"/>
     <mergeCell ref="W1:X1"/>
     <mergeCell ref="U1:V1"/>
     <mergeCell ref="C1"/>
@@ -17867,6 +17956,7 @@
     <mergeCell ref="A1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -17920,7 +18010,7 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="76" t="n">
+      <c r="A2" s="86" t="n">
         <v>33</v>
       </c>
       <c r="B2" s="77" t="inlineStr">
@@ -17933,7 +18023,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D2" s="79" t="n">
+      <c r="D2" s="91" t="n">
         <v>18</v>
       </c>
       <c r="E2" s="78" t="inlineStr">
@@ -17948,7 +18038,7 @@
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="80" t="n">
+      <c r="A3" s="89" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="81" t="inlineStr">
@@ -17961,7 +18051,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D3" s="83" t="n">
+      <c r="D3" s="92" t="n">
         <v>18</v>
       </c>
       <c r="E3" s="82" t="inlineStr">
@@ -17976,7 +18066,7 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="76" t="n">
+      <c r="A4" s="86" t="n">
         <v>22</v>
       </c>
       <c r="B4" s="77" t="inlineStr">
@@ -17989,7 +18079,7 @@
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="D4" s="79" t="n">
+      <c r="D4" s="91" t="n">
         <v>18</v>
       </c>
       <c r="E4" s="78" t="inlineStr">
@@ -18004,7 +18094,7 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="80" t="n">
+      <c r="A5" s="89" t="n">
         <v>16</v>
       </c>
       <c r="B5" s="81" t="inlineStr">
@@ -18017,7 +18107,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D5" s="83" t="n">
+      <c r="D5" s="92" t="n">
         <v>18</v>
       </c>
       <c r="E5" s="82" t="inlineStr">
@@ -18032,7 +18122,7 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="76" t="n">
+      <c r="A6" s="86" t="n">
         <v>26</v>
       </c>
       <c r="B6" s="77" t="inlineStr">
@@ -18045,7 +18135,7 @@
           <t>UK</t>
         </is>
       </c>
-      <c r="D6" s="79" t="n">
+      <c r="D6" s="91" t="n">
         <v>18</v>
       </c>
       <c r="E6" s="78" t="inlineStr">
@@ -18060,7 +18150,7 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="80" t="n">
+      <c r="A7" s="89" t="n">
         <v>14</v>
       </c>
       <c r="B7" s="81" t="inlineStr">
@@ -18088,7 +18178,7 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="76" t="n">
+      <c r="A8" s="86" t="n">
         <v>3</v>
       </c>
       <c r="B8" s="77" t="inlineStr">
@@ -18116,7 +18206,7 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="80" t="n">
+      <c r="A9" s="89" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="81" t="inlineStr">
@@ -18144,7 +18234,7 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="76" t="n">
+      <c r="A10" s="86" t="n">
         <v>37</v>
       </c>
       <c r="B10" s="77" t="inlineStr">
@@ -18172,7 +18262,7 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="80" t="n">
+      <c r="A11" s="89" t="n">
         <v>36</v>
       </c>
       <c r="B11" s="81" t="inlineStr">
@@ -18200,7 +18290,7 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="76" t="n">
+      <c r="A12" s="86" t="n">
         <v>9</v>
       </c>
       <c r="B12" s="77" t="inlineStr">
@@ -18228,7 +18318,7 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="80" t="n">
+      <c r="A13" s="89" t="n">
         <v>17</v>
       </c>
       <c r="B13" s="81" t="inlineStr">
@@ -18256,7 +18346,7 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="76" t="n">
+      <c r="A14" s="86" t="n">
         <v>25</v>
       </c>
       <c r="B14" s="77" t="inlineStr">
@@ -18284,7 +18374,7 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="80" t="n">
+      <c r="A15" s="89" t="n">
         <v>45</v>
       </c>
       <c r="B15" s="81" t="inlineStr">
@@ -18312,7 +18402,7 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="76" t="n">
+      <c r="A16" s="86" t="n">
         <v>53</v>
       </c>
       <c r="B16" s="77" t="inlineStr">
@@ -18340,7 +18430,7 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="80" t="n">
+      <c r="A17" s="89" t="n">
         <v>30</v>
       </c>
       <c r="B17" s="81" t="inlineStr">
@@ -18368,7 +18458,7 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="76" t="n">
+      <c r="A18" s="86" t="n">
         <v>31</v>
       </c>
       <c r="B18" s="77" t="inlineStr">
@@ -18396,7 +18486,7 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="80" t="n">
+      <c r="A19" s="89" t="n">
         <v>49</v>
       </c>
       <c r="B19" s="81" t="inlineStr">
@@ -18424,7 +18514,7 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="76" t="n">
+      <c r="A20" s="86" t="n">
         <v>68</v>
       </c>
       <c r="B20" s="77" t="inlineStr">
@@ -18452,7 +18542,7 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="80" t="n">
+      <c r="A21" s="89" t="n">
         <v>46</v>
       </c>
       <c r="B21" s="81" t="inlineStr">
@@ -18480,7 +18570,7 @@
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="76" t="n">
+      <c r="A22" s="86" t="n">
         <v>81</v>
       </c>
       <c r="B22" s="77" t="inlineStr">
@@ -18508,7 +18598,7 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="80" t="n">
+      <c r="A23" s="89" t="n">
         <v>19</v>
       </c>
       <c r="B23" s="81" t="inlineStr">
@@ -18536,7 +18626,7 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="76" t="n">
+      <c r="A24" s="86" t="n">
         <v>18</v>
       </c>
       <c r="B24" s="77" t="inlineStr">
@@ -18564,7 +18654,7 @@
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="80" t="n">
+      <c r="A25" s="89" t="n">
         <v>8</v>
       </c>
       <c r="B25" s="81" t="inlineStr">
@@ -18592,7 +18682,7 @@
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="76" t="n">
+      <c r="A26" s="86" t="n">
         <v>12</v>
       </c>
       <c r="B26" s="77" t="inlineStr">
@@ -18620,7 +18710,7 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="80" t="n">
+      <c r="A27" s="89" t="n">
         <v>46</v>
       </c>
       <c r="B27" s="81" t="inlineStr">
@@ -18648,7 +18738,7 @@
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="76" t="n">
+      <c r="A28" s="86" t="n">
         <v>88</v>
       </c>
       <c r="B28" s="77" t="inlineStr">
@@ -18676,7 +18766,7 @@
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="80" t="n">
+      <c r="A29" s="89" t="n">
         <v>97</v>
       </c>
       <c r="B29" s="81" t="inlineStr">
@@ -18704,7 +18794,7 @@
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="76" t="n">
+      <c r="A30" s="86" t="n">
         <v>83</v>
       </c>
       <c r="B30" s="77" t="inlineStr">
@@ -18732,7 +18822,7 @@
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="80" t="n">
+      <c r="A31" s="89" t="n">
         <v>7</v>
       </c>
       <c r="B31" s="81" t="inlineStr">
@@ -18760,7 +18850,7 @@
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="76" t="n">
+      <c r="A32" s="86" t="n">
         <v>51</v>
       </c>
       <c r="B32" s="77" t="inlineStr">
@@ -18788,7 +18878,7 @@
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="80" t="n">
+      <c r="A33" s="89" t="n">
         <v>53</v>
       </c>
       <c r="B33" s="81" t="inlineStr">
@@ -18816,7 +18906,7 @@
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="76" t="n">
+      <c r="A34" s="86" t="n">
         <v>76</v>
       </c>
       <c r="B34" s="77" t="inlineStr">
@@ -18844,7 +18934,7 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="80" t="n">
+      <c r="A35" s="89" t="n">
         <v>31</v>
       </c>
       <c r="B35" s="81" t="inlineStr">
@@ -18872,7 +18962,7 @@
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
-      <c r="A36" s="76" t="n">
+      <c r="A36" s="86" t="n">
         <v>20</v>
       </c>
       <c r="B36" s="77" t="inlineStr">
@@ -18900,7 +18990,7 @@
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="80" t="n">
+      <c r="A37" s="89" t="n">
         <v>55</v>
       </c>
       <c r="B37" s="81" t="inlineStr">
@@ -18928,7 +19018,7 @@
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="76" t="n">
+      <c r="A38" s="86" t="n">
         <v>56</v>
       </c>
       <c r="B38" s="77" t="inlineStr">
@@ -18956,7 +19046,7 @@
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="80" t="n">
+      <c r="A39" s="89" t="n">
         <v>24</v>
       </c>
       <c r="B39" s="81" t="inlineStr">
@@ -18984,7 +19074,7 @@
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="76" t="n">
+      <c r="A40" s="86" t="n">
         <v>79</v>
       </c>
       <c r="B40" s="77" t="inlineStr">
@@ -19012,7 +19102,7 @@
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="80" t="n">
+      <c r="A41" s="89" t="n">
         <v>76</v>
       </c>
       <c r="B41" s="81" t="inlineStr">
@@ -19040,7 +19130,7 @@
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
-      <c r="A42" s="76" t="n">
+      <c r="A42" s="86" t="n">
         <v>80</v>
       </c>
       <c r="B42" s="77" t="inlineStr">
@@ -19068,7 +19158,7 @@
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
-      <c r="A43" s="80" t="n">
+      <c r="A43" s="89" t="n">
         <v>1</v>
       </c>
       <c r="B43" s="81" t="inlineStr">
@@ -19096,7 +19186,7 @@
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
-      <c r="A44" s="76" t="n">
+      <c r="A44" s="86" t="n">
         <v>10</v>
       </c>
       <c r="B44" s="77" t="inlineStr">
@@ -19124,7 +19214,7 @@
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
-      <c r="A45" s="80" t="n">
+      <c r="A45" s="89" t="n">
         <v>11</v>
       </c>
       <c r="B45" s="81" t="inlineStr">
@@ -19152,7 +19242,7 @@
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
-      <c r="A46" s="76" t="n">
+      <c r="A46" s="86" t="n">
         <v>14</v>
       </c>
       <c r="B46" s="77" t="inlineStr">
@@ -19180,7 +19270,7 @@
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
-      <c r="A47" s="80" t="n">
+      <c r="A47" s="89" t="n">
         <v>98</v>
       </c>
       <c r="B47" s="81" t="inlineStr">
@@ -19208,7 +19298,7 @@
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
-      <c r="A48" s="76" t="n">
+      <c r="A48" s="86" t="n">
         <v>28</v>
       </c>
       <c r="B48" s="77" t="inlineStr">
@@ -19236,7 +19326,7 @@
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
-      <c r="A49" s="80" t="n">
+      <c r="A49" s="89" t="n">
         <v>88</v>
       </c>
       <c r="B49" s="81" t="inlineStr">
@@ -19249,7 +19339,7 @@
           <t>Singapore</t>
         </is>
       </c>
-      <c r="D49" s="80" t="n">
+      <c r="D49" s="89" t="n">
         <v>13</v>
       </c>
       <c r="E49" s="82" t="inlineStr">
@@ -19264,7 +19354,7 @@
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
-      <c r="A50" s="76" t="n">
+      <c r="A50" s="86" t="n">
         <v>13</v>
       </c>
       <c r="B50" s="77" t="inlineStr">
@@ -19277,7 +19367,7 @@
           <t>France</t>
         </is>
       </c>
-      <c r="D50" s="76" t="n">
+      <c r="D50" s="86" t="n">
         <v>13</v>
       </c>
       <c r="E50" s="78" t="inlineStr">
@@ -19292,7 +19382,7 @@
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
-      <c r="A51" s="80" t="n">
+      <c r="A51" s="89" t="n">
         <v>72</v>
       </c>
       <c r="B51" s="81" t="inlineStr">
@@ -19305,7 +19395,7 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="D51" s="80" t="n">
+      <c r="D51" s="89" t="n">
         <v>13</v>
       </c>
       <c r="E51" s="82" t="inlineStr">
@@ -19320,7 +19410,7 @@
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
-      <c r="A52" s="76" t="n">
+      <c r="A52" s="86" t="n">
         <v>35</v>
       </c>
       <c r="B52" s="77" t="inlineStr">
@@ -19333,7 +19423,7 @@
           <t>Denmark</t>
         </is>
       </c>
-      <c r="D52" s="76" t="n">
+      <c r="D52" s="86" t="n">
         <v>13</v>
       </c>
       <c r="E52" s="78" t="inlineStr">
@@ -19348,7 +19438,7 @@
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
-      <c r="A53" s="80" t="n">
+      <c r="A53" s="89" t="n">
         <v>26</v>
       </c>
       <c r="B53" s="81" t="inlineStr">
@@ -19361,7 +19451,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D53" s="80" t="n">
+      <c r="D53" s="89" t="n">
         <v>13</v>
       </c>
       <c r="E53" s="82" t="inlineStr">
@@ -19376,7 +19466,7 @@
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
-      <c r="A54" s="76" t="n">
+      <c r="A54" s="86" t="n">
         <v>44</v>
       </c>
       <c r="B54" s="77" t="inlineStr">
@@ -19389,7 +19479,7 @@
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="D54" s="76" t="n">
+      <c r="D54" s="86" t="n">
         <v>13</v>
       </c>
       <c r="E54" s="78" t="inlineStr">
@@ -19404,7 +19494,7 @@
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
-      <c r="A55" s="80" t="n">
+      <c r="A55" s="89" t="n">
         <v>62</v>
       </c>
       <c r="B55" s="81" t="inlineStr">
@@ -19417,7 +19507,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D55" s="80" t="n">
+      <c r="D55" s="89" t="n">
         <v>13</v>
       </c>
       <c r="E55" s="82" t="inlineStr">
@@ -19432,7 +19522,7 @@
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
-      <c r="A56" s="76" t="n">
+      <c r="A56" s="86" t="n">
         <v>61</v>
       </c>
       <c r="B56" s="77" t="inlineStr">
@@ -19445,7 +19535,7 @@
           <t>UK</t>
         </is>
       </c>
-      <c r="D56" s="76" t="n">
+      <c r="D56" s="86" t="n">
         <v>12</v>
       </c>
       <c r="E56" s="78" t="inlineStr">
@@ -19460,7 +19550,7 @@
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
-      <c r="A57" s="80" t="n">
+      <c r="A57" s="89" t="n">
         <v>91</v>
       </c>
       <c r="B57" s="81" t="inlineStr">
@@ -19473,7 +19563,7 @@
           <t>Belgium</t>
         </is>
       </c>
-      <c r="D57" s="80" t="n">
+      <c r="D57" s="89" t="n">
         <v>12</v>
       </c>
       <c r="E57" s="82" t="inlineStr">
@@ -19488,7 +19578,7 @@
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
-      <c r="A58" s="76" t="n">
+      <c r="A58" s="86" t="n">
         <v>76</v>
       </c>
       <c r="B58" s="77" t="inlineStr">
@@ -19501,7 +19591,7 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="D58" s="76" t="n">
+      <c r="D58" s="86" t="n">
         <v>12</v>
       </c>
       <c r="E58" s="78" t="inlineStr">
@@ -19516,7 +19606,7 @@
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
-      <c r="A59" s="80" t="n">
+      <c r="A59" s="89" t="n">
         <v>67</v>
       </c>
       <c r="B59" s="81" t="inlineStr">
@@ -19529,7 +19619,7 @@
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="D59" s="80" t="n">
+      <c r="D59" s="89" t="n">
         <v>12</v>
       </c>
       <c r="E59" s="82" t="inlineStr">
@@ -19544,7 +19634,7 @@
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
-      <c r="A60" s="76" t="n">
+      <c r="A60" s="86" t="n">
         <v>65</v>
       </c>
       <c r="B60" s="77" t="inlineStr">
@@ -19557,7 +19647,7 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="D60" s="76" t="n">
+      <c r="D60" s="86" t="n">
         <v>12</v>
       </c>
       <c r="E60" s="78" t="inlineStr">
@@ -19572,7 +19662,7 @@
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
-      <c r="A61" s="80" t="n">
+      <c r="A61" s="89" t="n">
         <v>46</v>
       </c>
       <c r="B61" s="81" t="inlineStr">
@@ -19585,7 +19675,7 @@
           <t>Japan</t>
         </is>
       </c>
-      <c r="D61" s="80" t="n">
+      <c r="D61" s="89" t="n">
         <v>12</v>
       </c>
       <c r="E61" s="82" t="inlineStr">
@@ -19600,7 +19690,7 @@
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
-      <c r="A62" s="76" t="n">
+      <c r="A62" s="86" t="n">
         <v>38</v>
       </c>
       <c r="B62" s="77" t="inlineStr">
@@ -19613,7 +19703,7 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="D62" s="76" t="n">
+      <c r="D62" s="86" t="n">
         <v>12</v>
       </c>
       <c r="E62" s="78" t="inlineStr">
@@ -19628,7 +19718,7 @@
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
-      <c r="A63" s="80" t="n">
+      <c r="A63" s="89" t="n">
         <v>40</v>
       </c>
       <c r="B63" s="81" t="inlineStr">
@@ -19641,7 +19731,7 @@
           <t>China</t>
         </is>
       </c>
-      <c r="D63" s="80" t="n">
+      <c r="D63" s="89" t="n">
         <v>12</v>
       </c>
       <c r="E63" s="82" t="inlineStr">
@@ -19656,7 +19746,7 @@
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
-      <c r="A64" s="76" t="n">
+      <c r="A64" s="86" t="n">
         <v>99</v>
       </c>
       <c r="B64" s="77" t="inlineStr">
@@ -19669,7 +19759,7 @@
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="D64" s="76" t="n">
+      <c r="D64" s="86" t="n">
         <v>11</v>
       </c>
       <c r="E64" s="78" t="inlineStr">
@@ -19684,7 +19774,7 @@
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
-      <c r="A65" s="80" t="n">
+      <c r="A65" s="89" t="n">
         <v>62</v>
       </c>
       <c r="B65" s="81" t="inlineStr">
@@ -19697,7 +19787,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D65" s="80" t="n">
+      <c r="D65" s="89" t="n">
         <v>11</v>
       </c>
       <c r="E65" s="82" t="inlineStr">
@@ -19712,7 +19802,7 @@
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
-      <c r="A66" s="76" t="n">
+      <c r="A66" s="86" t="n">
         <v>4</v>
       </c>
       <c r="B66" s="77" t="inlineStr">
@@ -19725,7 +19815,7 @@
           <t>UK</t>
         </is>
       </c>
-      <c r="D66" s="76" t="n">
+      <c r="D66" s="86" t="n">
         <v>11</v>
       </c>
       <c r="E66" s="78" t="inlineStr">
@@ -19740,7 +19830,7 @@
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
-      <c r="A67" s="80" t="n">
+      <c r="A67" s="89" t="n">
         <v>6</v>
       </c>
       <c r="B67" s="81" t="inlineStr">
@@ -19753,7 +19843,7 @@
           <t>UK</t>
         </is>
       </c>
-      <c r="D67" s="80" t="n">
+      <c r="D67" s="89" t="n">
         <v>11</v>
       </c>
       <c r="E67" s="82" t="inlineStr">
@@ -19768,7 +19858,7 @@
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
-      <c r="A68" s="76" t="n">
+      <c r="A68" s="86" t="n">
         <v>34</v>
       </c>
       <c r="B68" s="77" t="inlineStr">
@@ -19781,7 +19871,7 @@
           <t>France</t>
         </is>
       </c>
-      <c r="D68" s="76" t="n">
+      <c r="D68" s="86" t="n">
         <v>11</v>
       </c>
       <c r="E68" s="78" t="inlineStr">
@@ -19796,7 +19886,7 @@
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
-      <c r="A69" s="80" t="n">
+      <c r="A69" s="89" t="n">
         <v>42</v>
       </c>
       <c r="B69" s="81" t="inlineStr">
@@ -19809,7 +19899,7 @@
           <t>Germany</t>
         </is>
       </c>
-      <c r="D69" s="80" t="n">
+      <c r="D69" s="89" t="n">
         <v>11</v>
       </c>
       <c r="E69" s="82" t="inlineStr">
@@ -19824,7 +19914,7 @@
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
-      <c r="A70" s="76" t="n">
+      <c r="A70" s="86" t="n">
         <v>70</v>
       </c>
       <c r="B70" s="77" t="inlineStr">
@@ -19837,7 +19927,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D70" s="76" t="n">
+      <c r="D70" s="86" t="n">
         <v>11</v>
       </c>
       <c r="E70" s="78" t="inlineStr">
@@ -19852,7 +19942,7 @@
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
-      <c r="A71" s="80" t="n">
+      <c r="A71" s="89" t="n">
         <v>41</v>
       </c>
       <c r="B71" s="81" t="inlineStr">
@@ -19865,7 +19955,7 @@
           <t>China</t>
         </is>
       </c>
-      <c r="D71" s="80" t="n">
+      <c r="D71" s="89" t="n">
         <v>11</v>
       </c>
       <c r="E71" s="82" t="inlineStr">
@@ -19880,7 +19970,7 @@
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
-      <c r="A72" s="76" t="n">
+      <c r="A72" s="86" t="n">
         <v>73</v>
       </c>
       <c r="B72" s="77" t="inlineStr">
@@ -19893,7 +19983,7 @@
           <t>China</t>
         </is>
       </c>
-      <c r="D72" s="76" t="n">
+      <c r="D72" s="86" t="n">
         <v>11</v>
       </c>
       <c r="E72" s="78" t="inlineStr">
@@ -19908,7 +19998,7 @@
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
-      <c r="A73" s="80" t="n">
+      <c r="A73" s="89" t="n">
         <v>92</v>
       </c>
       <c r="B73" s="81" t="inlineStr">
@@ -19921,7 +20011,7 @@
           <t>China</t>
         </is>
       </c>
-      <c r="D73" s="80" t="n">
+      <c r="D73" s="89" t="n">
         <v>10</v>
       </c>
       <c r="E73" s="82" t="inlineStr">
@@ -19936,7 +20026,7 @@
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
-      <c r="A74" s="76" t="n">
+      <c r="A74" s="86" t="n">
         <v>88</v>
       </c>
       <c r="B74" s="77" t="inlineStr">
@@ -19949,7 +20039,7 @@
           <t>Israel</t>
         </is>
       </c>
-      <c r="D74" s="76" t="n">
+      <c r="D74" s="86" t="n">
         <v>10</v>
       </c>
       <c r="E74" s="78" t="inlineStr">
@@ -19964,7 +20054,7 @@
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
-      <c r="A75" s="80" t="n">
+      <c r="A75" s="89" t="n">
         <v>85</v>
       </c>
       <c r="B75" s="81" t="inlineStr">
@@ -19977,7 +20067,7 @@
           <t>Denmark</t>
         </is>
       </c>
-      <c r="D75" s="80" t="n">
+      <c r="D75" s="89" t="n">
         <v>10</v>
       </c>
       <c r="E75" s="82" t="inlineStr">
@@ -19992,7 +20082,7 @@
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
-      <c r="A76" s="76" t="n">
+      <c r="A76" s="86" t="n">
         <v>43</v>
       </c>
       <c r="B76" s="77" t="inlineStr">
@@ -20005,7 +20095,7 @@
           <t>France</t>
         </is>
       </c>
-      <c r="D76" s="76" t="n">
+      <c r="D76" s="86" t="n">
         <v>10</v>
       </c>
       <c r="E76" s="78" t="inlineStr">
@@ -20020,7 +20110,7 @@
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
-      <c r="A77" s="80" t="n">
+      <c r="A77" s="89" t="n">
         <v>56</v>
       </c>
       <c r="B77" s="81" t="inlineStr">
@@ -20033,7 +20123,7 @@
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="D77" s="80" t="n">
+      <c r="D77" s="89" t="n">
         <v>10</v>
       </c>
       <c r="E77" s="82" t="inlineStr">
@@ -20048,7 +20138,7 @@
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
-      <c r="A78" s="76" t="n">
+      <c r="A78" s="86" t="n">
         <v>65</v>
       </c>
       <c r="B78" s="77" t="inlineStr">
@@ -20061,7 +20151,7 @@
           <t>China</t>
         </is>
       </c>
-      <c r="D78" s="76" t="n">
+      <c r="D78" s="86" t="n">
         <v>10</v>
       </c>
       <c r="E78" s="78" t="inlineStr">
@@ -20076,7 +20166,7 @@
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
-      <c r="A79" s="80" t="n">
+      <c r="A79" s="89" t="n">
         <v>64</v>
       </c>
       <c r="B79" s="81" t="inlineStr">
@@ -20089,7 +20179,7 @@
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="D79" s="80" t="n">
+      <c r="D79" s="89" t="n">
         <v>10</v>
       </c>
       <c r="E79" s="82" t="inlineStr">
@@ -20104,7 +20194,7 @@
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
-      <c r="A80" s="76" t="n">
+      <c r="A80" s="86" t="n">
         <v>96</v>
       </c>
       <c r="B80" s="77" t="inlineStr">
@@ -20117,7 +20207,7 @@
           <t>China</t>
         </is>
       </c>
-      <c r="D80" s="76" t="n">
+      <c r="D80" s="86" t="n">
         <v>10</v>
       </c>
       <c r="E80" s="78" t="inlineStr">
@@ -20132,7 +20222,7 @@
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
-      <c r="A81" s="80" t="n">
+      <c r="A81" s="89" t="n">
         <v>58</v>
       </c>
       <c r="B81" s="81" t="inlineStr">
@@ -20145,7 +20235,7 @@
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="D81" s="80" t="n">
+      <c r="D81" s="89" t="n">
         <v>9</v>
       </c>
       <c r="E81" s="82" t="inlineStr">
@@ -20160,7 +20250,7 @@
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
-      <c r="A82" s="76" t="n">
+      <c r="A82" s="86" t="n">
         <v>39</v>
       </c>
       <c r="B82" s="77" t="inlineStr">
@@ -20173,7 +20263,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D82" s="76" t="n">
+      <c r="D82" s="86" t="n">
         <v>9</v>
       </c>
       <c r="E82" s="78" t="inlineStr">
@@ -20188,7 +20278,7 @@
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
-      <c r="A83" s="80" t="n">
+      <c r="A83" s="89" t="n">
         <v>93</v>
       </c>
       <c r="B83" s="81" t="inlineStr">
@@ -20201,7 +20291,7 @@
           <t>Sweden</t>
         </is>
       </c>
-      <c r="D83" s="80" t="n">
+      <c r="D83" s="89" t="n">
         <v>9</v>
       </c>
       <c r="E83" s="82" t="inlineStr">
@@ -20216,7 +20306,7 @@
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
-      <c r="A84" s="76" t="n">
+      <c r="A84" s="86" t="n">
         <v>71</v>
       </c>
       <c r="B84" s="77" t="inlineStr">
@@ -20229,7 +20319,7 @@
           <t>Israel</t>
         </is>
       </c>
-      <c r="D84" s="76" t="n">
+      <c r="D84" s="86" t="n">
         <v>9</v>
       </c>
       <c r="E84" s="78" t="inlineStr">
@@ -20244,7 +20334,7 @@
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
-      <c r="A85" s="80" t="n">
+      <c r="A85" s="89" t="n">
         <v>23</v>
       </c>
       <c r="B85" s="81" t="inlineStr">
@@ -20257,7 +20347,7 @@
           <t>China</t>
         </is>
       </c>
-      <c r="D85" s="80" t="n">
+      <c r="D85" s="89" t="n">
         <v>9</v>
       </c>
       <c r="E85" s="82" t="inlineStr">
@@ -20272,7 +20362,7 @@
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
-      <c r="A86" s="76" t="n">
+      <c r="A86" s="86" t="n">
         <v>94</v>
       </c>
       <c r="B86" s="77" t="inlineStr">
@@ -20285,7 +20375,7 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D86" s="76" t="n">
+      <c r="D86" s="86" t="n">
         <v>9</v>
       </c>
       <c r="E86" s="78" t="inlineStr">
@@ -20300,7 +20390,7 @@
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
-      <c r="A87" s="80" t="n">
+      <c r="A87" s="89" t="n">
         <v>81</v>
       </c>
       <c r="B87" s="81" t="inlineStr">
@@ -20313,7 +20403,7 @@
           <t>China</t>
         </is>
       </c>
-      <c r="D87" s="80" t="n">
+      <c r="D87" s="89" t="n">
         <v>9</v>
       </c>
       <c r="E87" s="82" t="inlineStr">
@@ -20328,7 +20418,7 @@
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
-      <c r="A88" s="76" t="n">
+      <c r="A88" s="86" t="n">
         <v>83</v>
       </c>
       <c r="B88" s="77" t="inlineStr">
@@ -20341,7 +20431,7 @@
           <t>Norway</t>
         </is>
       </c>
-      <c r="D88" s="76" t="n">
+      <c r="D88" s="86" t="n">
         <v>9</v>
       </c>
       <c r="E88" s="78" t="inlineStr">
@@ -20356,7 +20446,7 @@
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
-      <c r="A89" s="80" t="n">
+      <c r="A89" s="89" t="n">
         <v>87</v>
       </c>
       <c r="B89" s="81" t="inlineStr">
@@ -20369,7 +20459,7 @@
           <t>China</t>
         </is>
       </c>
-      <c r="D89" s="80" t="n">
+      <c r="D89" s="89" t="n">
         <v>9</v>
       </c>
       <c r="E89" s="82" t="inlineStr">
@@ -20384,7 +20474,7 @@
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
-      <c r="A90" s="76" t="n">
+      <c r="A90" s="86" t="n">
         <v>60</v>
       </c>
       <c r="B90" s="77" t="inlineStr">
@@ -20397,7 +20487,7 @@
           <t>France</t>
         </is>
       </c>
-      <c r="D90" s="76" t="n">
+      <c r="D90" s="86" t="n">
         <v>9</v>
       </c>
       <c r="E90" s="78" t="inlineStr">
@@ -20412,7 +20502,7 @@
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
-      <c r="A91" s="80" t="n">
+      <c r="A91" s="89" t="n">
         <v>51</v>
       </c>
       <c r="B91" s="81" t="inlineStr">
@@ -20425,7 +20515,7 @@
           <t>Germany</t>
         </is>
       </c>
-      <c r="D91" s="80" t="n">
+      <c r="D91" s="89" t="n">
         <v>8</v>
       </c>
       <c r="E91" s="82" t="inlineStr">
@@ -20440,7 +20530,7 @@
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
-      <c r="A92" s="76" t="n">
+      <c r="A92" s="86" t="n">
         <v>75</v>
       </c>
       <c r="B92" s="77" t="inlineStr">
@@ -20453,7 +20543,7 @@
           <t>China</t>
         </is>
       </c>
-      <c r="D92" s="76" t="n">
+      <c r="D92" s="86" t="n">
         <v>8</v>
       </c>
       <c r="E92" s="78" t="inlineStr">
@@ -20468,7 +20558,7 @@
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
-      <c r="A93" s="80" t="n">
+      <c r="A93" s="89" t="n">
         <v>73</v>
       </c>
       <c r="B93" s="81" t="inlineStr">
@@ -20481,7 +20571,7 @@
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="D93" s="80" t="n">
+      <c r="D93" s="89" t="n">
         <v>8</v>
       </c>
       <c r="E93" s="82" t="inlineStr">
@@ -20496,7 +20586,7 @@
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
-      <c r="A94" s="76" t="n">
+      <c r="A94" s="86" t="n">
         <v>100</v>
       </c>
       <c r="B94" s="77" t="inlineStr">
@@ -20509,7 +20599,7 @@
           <t>Sweden</t>
         </is>
       </c>
-      <c r="D94" s="76" t="n">
+      <c r="D94" s="86" t="n">
         <v>8</v>
       </c>
       <c r="E94" s="78" t="inlineStr">
@@ -20524,7 +20614,7 @@
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
-      <c r="A95" s="80" t="n">
+      <c r="A95" s="89" t="n">
         <v>94</v>
       </c>
       <c r="B95" s="81" t="inlineStr">
@@ -20537,7 +20627,7 @@
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="D95" s="80" t="n">
+      <c r="D95" s="89" t="n">
         <v>7</v>
       </c>
       <c r="E95" s="82" t="inlineStr">
@@ -20552,7 +20642,7 @@
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
-      <c r="A96" s="76" t="n">
+      <c r="A96" s="86" t="n">
         <v>68</v>
       </c>
       <c r="B96" s="77" t="inlineStr">
@@ -20565,7 +20655,7 @@
           <t>Germany</t>
         </is>
       </c>
-      <c r="D96" s="76" t="n">
+      <c r="D96" s="86" t="n">
         <v>7</v>
       </c>
       <c r="E96" s="78" t="inlineStr">
@@ -20580,7 +20670,7 @@
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
-      <c r="A97" s="80" t="n">
+      <c r="A97" s="89" t="n">
         <v>21</v>
       </c>
       <c r="B97" s="81" t="inlineStr">
@@ -20593,7 +20683,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D97" s="80" t="n">
+      <c r="D97" s="89" t="n">
         <v>5</v>
       </c>
       <c r="E97" s="82" t="inlineStr">
@@ -20608,7 +20698,7 @@
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">
-      <c r="A98" s="76" t="n">
+      <c r="A98" s="86" t="n">
         <v>29</v>
       </c>
       <c r="B98" s="77" t="inlineStr">
@@ -20621,7 +20711,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D98" s="76" t="n">
+      <c r="D98" s="86" t="n">
         <v>4</v>
       </c>
       <c r="E98" s="78" t="inlineStr">
@@ -20636,7 +20726,7 @@
       </c>
     </row>
     <row r="99" ht="15" customHeight="1">
-      <c r="A99" s="80" t="n">
+      <c r="A99" s="89" t="n">
         <v>86</v>
       </c>
       <c r="B99" s="81" t="inlineStr">
@@ -20649,7 +20739,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D99" s="80" t="n">
+      <c r="D99" s="89" t="n">
         <v>3</v>
       </c>
       <c r="E99" s="82" t="inlineStr">
@@ -20664,7 +20754,7 @@
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
-      <c r="A100" s="76" t="n">
+      <c r="A100" s="86" t="n">
         <v>58</v>
       </c>
       <c r="B100" s="77" t="inlineStr">
@@ -20677,7 +20767,7 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D100" s="76" t="n">
+      <c r="D100" s="86" t="n">
         <v>3</v>
       </c>
       <c r="E100" s="78" t="inlineStr">
@@ -20692,7 +20782,7 @@
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
-      <c r="A101" s="80" t="n">
+      <c r="A101" s="89" t="n">
         <v>50</v>
       </c>
       <c r="B101" s="81" t="inlineStr">
@@ -20705,7 +20795,7 @@
           <t>Sweden</t>
         </is>
       </c>
-      <c r="D101" s="80" t="n">
+      <c r="D101" s="89" t="n">
         <v>3</v>
       </c>
       <c r="E101" s="82" t="inlineStr">

</xml_diff>